<commit_message>
doc: fin del apartado teórico del curso de Dalto donde se trataron los temas de normalización y cardinalidad para entender en profundidad las relaciones entre tablas y cómo optimizarla desde su creación
</commit_message>
<xml_diff>
--- a/curso-sql/soy-dalto/resources/excel/Gráficos.xlsx
+++ b/curso-sql/soy-dalto/resources/excel/Gráficos.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\Documents\Devs\desarrollo_fundamentos_transversales\curso-sql\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\Documents\Devs\cursos\curso-sql\soy-dalto\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DD9E0AB-6380-4A78-BF12-4C7FC254E204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F04659B-2D5C-490C-92C7-AF17C4430322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{58D3E8CE-0E43-4FF8-851A-296749E05404}"/>
   </bookViews>
   <sheets>
-    <sheet name="Relación entre tablas" sheetId="1" r:id="rId1"/>
+    <sheet name="Cardinalidad" sheetId="2" r:id="rId1"/>
+    <sheet name="Relación entre tablas" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
   <si>
     <t>turnos_medicos</t>
   </si>
@@ -78,6 +79,150 @@
   </si>
   <si>
     <t>RELACIÓN ENTRE TABLAS UNO A MUCHOS</t>
+  </si>
+  <si>
+    <t>CARDINALIDAD - DB NORTHWIND</t>
+  </si>
+  <si>
+    <t>Customers</t>
+  </si>
+  <si>
+    <t>CustomerID</t>
+  </si>
+  <si>
+    <t>CustomerName</t>
+  </si>
+  <si>
+    <t>ContactName</t>
+  </si>
+  <si>
+    <t>Adderss</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>PostalCode</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CustomerID </t>
+  </si>
+  <si>
+    <t>Employess</t>
+  </si>
+  <si>
+    <t>EmployeeID</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>BirthDate</t>
+  </si>
+  <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Shippers</t>
+  </si>
+  <si>
+    <t>ShipperID</t>
+  </si>
+  <si>
+    <t>ShipperName</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>OrderID</t>
+  </si>
+  <si>
+    <t>OrderDate</t>
+  </si>
+  <si>
+    <t>OrderDetails</t>
+  </si>
+  <si>
+    <t>OderDetailID</t>
+  </si>
+  <si>
+    <t>ProductID</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>SupplierID</t>
+  </si>
+  <si>
+    <t>CategoryID</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Suppliers</t>
+  </si>
+  <si>
+    <t>SupplierName</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>CategoryName</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>One</t>
+  </si>
+  <si>
+    <t>Many</t>
+  </si>
+  <si>
+    <t>One (and only one)</t>
+  </si>
+  <si>
+    <t>Zero or one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1:n </t>
+  </si>
+  <si>
+    <t>n:1</t>
+  </si>
+  <si>
+    <t>1:1</t>
+  </si>
+  <si>
+    <t>n:m</t>
   </si>
 </sst>
 </file>
@@ -121,7 +266,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -144,20 +289,136 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -176,6 +437,1858 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>133351</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="94" name="Rectángulo 93">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{111AF591-6598-4A48-82D0-11ED39F0C488}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6991350" y="2628900"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>866778</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>152398</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="74" name="Conector: angular 73">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43471949-9077-4006-97FD-32D8B8C6B35E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000" flipV="1">
+          <a:off x="6962778" y="904875"/>
+          <a:ext cx="1533523" cy="1485898"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>752475</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>85726</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="68" name="Rectángulo 67">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7F31142-41DE-46F2-B973-68EFD78D1039}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4048125" y="1914525"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>95251</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="67" name="Rectángulo 66">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0AEAC72-1775-448B-9453-F6C1B6EE7EEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3552825" y="1733550"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>171451</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="59" name="Rectángulo 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{902F4256-52E6-4E6D-AA98-6552B8972693}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2352675" y="2857500"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>485775</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>714375</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>95251</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="58" name="Rectángulo 57">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2D052FD-CED9-47FF-9FAF-75DC6F643AF8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2343150" y="2352675"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="6" name="Conector recto 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2768578-7093-4460-9808-25874DF5B61D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2990850" y="5048250"/>
+          <a:ext cx="1419225" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="7" name="Conector recto 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3AF09CF9-4D6A-49DC-9AC2-B1585BFDAF6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2981325" y="5410200"/>
+          <a:ext cx="1419225" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="8" name="Conector recto 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{096FE8C4-EC51-45FA-8E57-81B7913A6ABB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2990850" y="5743575"/>
+          <a:ext cx="1419225" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="9" name="Conector recto 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B8A8F42-19CC-4878-A938-D5EC39455C01}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3000375" y="6134100"/>
+          <a:ext cx="1419225" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>76884</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>94567</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="15" name="Conector recto 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3387ED43-315E-6DDB-635B-A42BD4AF5C1A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4257675" y="4944159"/>
+          <a:ext cx="0" cy="208183"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="16" name="Conector recto 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B107C1E-5921-49F1-8C35-7AC978024670}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4191000" y="5305425"/>
+          <a:ext cx="209550" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>657225</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="18" name="Conector recto 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C31FF8B3-E65D-47F8-9EF1-95FE644AF565}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4181475" y="5410200"/>
+          <a:ext cx="219075" cy="114300"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>10209</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>27892</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="28" name="Conector recto 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E99C8E0B-22DD-4297-81A3-A164CEAD28C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4248150" y="5639484"/>
+          <a:ext cx="0" cy="208183"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>10209</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>27892</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="29" name="Conector recto 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA781F54-C337-45A5-8ABB-2E4A9ADFED8C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4333875" y="5639484"/>
+          <a:ext cx="0" cy="208183"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>19734</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>37417</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="30" name="Conector recto 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0513DD2-7D45-4EE8-9E8F-6F79A52E0BEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4343400" y="6030009"/>
+          <a:ext cx="0" cy="208183"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>742950</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="Elipse 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{91293A6B-01E6-01AD-4051-D434C253E357}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4000500" y="6000750"/>
+          <a:ext cx="266700" cy="247650"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="dk1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-VE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="33" name="Conector: angular 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EF21439-C9F7-854A-D69F-D2858977BC44}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="990600" y="838200"/>
+          <a:ext cx="1638300" cy="1314450"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 49419"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="35" name="Conector: angular 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC222CE2-94C5-4434-8815-8AA42423ED8C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="981075" y="2333625"/>
+          <a:ext cx="1647825" cy="352425"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="45" name="Conector: angular 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{745DE048-95B5-4DB1-AC9F-B43E7F7E45CD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="990600" y="2828925"/>
+          <a:ext cx="1638300" cy="1438275"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>161926</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="54" name="Rectángulo 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17C6CCA7-D81A-4493-791C-7DCBB94168ED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1000125" y="609600"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>704850</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>57151</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="56" name="Rectángulo 55">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB355023-484A-4E8C-AEB8-CFBFA7EA5088}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2333625" y="1885950"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>200025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>180976</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="Rectángulo 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{308D93F0-0255-4F82-97C1-546ABA363263}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1019175" y="2438400"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>152401</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="Rectángulo 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98E2A099-E101-4F0F-AF4F-476ACB1E3791}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1028700" y="4029075"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="62" name="Conector: angular 61">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD5823E9-3C33-45D6-85E8-959C6471D133}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3533775" y="1952625"/>
+          <a:ext cx="752475" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1038226</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>104774</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="69" name="Conector: angular 68">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36429E21-BDCD-40E4-B8C1-5B991BD6F86E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000" flipV="1">
+          <a:off x="5324476" y="1962149"/>
+          <a:ext cx="771527" cy="371475"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>752475</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>76201</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="72" name="Rectángulo 71">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5565AA79-5EA2-48F5-8480-C4F23F344ABB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5857875" y="1714500"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>66676</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="73" name="Rectángulo 72">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94602F94-04C4-4256-A792-F2861331E583}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5353050" y="2085975"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>752475</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="90" name="Rectángulo 89">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55BF1C0B-08C1-4AD9-94C0-2148C37D7CB2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8258175" y="723900"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="91" name="Rectángulo 90">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8810E4D3-50BE-48F8-962C-C8E9C19C6DA7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6991350" y="2181225"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>n</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>752480</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>85723</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="92" name="Conector: angular 91">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18C4F619-4376-4B14-B57C-A209B5734A49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="6972301" y="2600325"/>
+          <a:ext cx="1514479" cy="438148"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>76201</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="95" name="Rectángulo 94">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF4EED14-4E28-427A-BAF2-D441275D7D5D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8229600" y="2809875"/>
+          <a:ext cx="228600" cy="219076"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-VE" sz="1100"/>
+            <a:t>1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -549,28 +2662,339 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A81E75-79BE-431C-BA62-8782E472CAA5}">
+  <dimension ref="A1:K32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="3" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="18"/>
+      <c r="D4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D11" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D24" s="9"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="11"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D25" s="12"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" s="14"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D26" s="12"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="14"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D27" s="12"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="H27" s="14"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D28" s="12"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="14"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D29" s="12"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="H29" s="14"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D30" s="12"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="14"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D31" s="12"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="H31" s="14"/>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D32" s="15"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38BD871B-7997-4787-8360-023FEFD0B2A1}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
     </row>
     <row r="3" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="D3" s="1" t="s">
+      <c r="B3" s="4"/>
+      <c r="D3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">

</xml_diff>